<commit_message>
Scrapper: 11.08.2026 08:50 – aktualizace výsledků
</commit_message>
<xml_diff>
--- a/vysledky.xlsx
+++ b/vysledky.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,6 +119,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -505,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I353"/>
+  <dimension ref="A1:I355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -15886,13 +15898,89 @@
       </c>
       <c r="I353" s="9" t="inlineStr"/>
     </row>
+    <row r="354" ht="18" customHeight="1">
+      <c r="A354" s="5" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B354" s="11" t="inlineStr">
+        <is>
+          <t>polar.cz</t>
+        </is>
+      </c>
+      <c r="C354" s="11" t="inlineStr">
+        <is>
+          <t>Ondřej Havelka a jeho Melody Makers / koncert</t>
+        </is>
+      </c>
+      <c r="D354" s="12" t="inlineStr">
+        <is>
+          <t>https://polar.cz/kam-vyrazit/moravskoslezsky-kraj/cely-ms-kraj/11000017180/ondrej-havelka-a-jeho-melody-makers--koncert</t>
+        </is>
+      </c>
+      <c r="E354" s="11" t="inlineStr"/>
+      <c r="F354" s="11" t="inlineStr">
+        <is>
+          <t>Jiné</t>
+        </is>
+      </c>
+      <c r="G354" s="11" t="inlineStr">
+        <is>
+          <t>11.08.2026 08:50</t>
+        </is>
+      </c>
+      <c r="H354" s="11" t="inlineStr"/>
+      <c r="I354" s="11" t="inlineStr"/>
+    </row>
+    <row r="355" ht="18" customHeight="1">
+      <c r="A355" s="8" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B355" s="13" t="inlineStr">
+        <is>
+          <t>polar.cz</t>
+        </is>
+      </c>
+      <c r="C355" s="13" t="inlineStr">
+        <is>
+          <t>Učitelé praktického vyučování (kromě pro žáky se speciálními vzdělávacími potřebami)</t>
+        </is>
+      </c>
+      <c r="D355" s="14" t="inlineStr">
+        <is>
+          <t>https://polar.cz/nabidka-prace/ostrava/detail/33291660710/ucitele-praktickeho-vyucovani-krome-pro-zaky-se-specialnimi-vzdelavacimi-potrebami</t>
+        </is>
+      </c>
+      <c r="E355" s="13" t="inlineStr"/>
+      <c r="F355" s="13" t="inlineStr">
+        <is>
+          <t>Jiné</t>
+        </is>
+      </c>
+      <c r="G355" s="13" t="inlineStr">
+        <is>
+          <t>11.08.2026 08:50</t>
+        </is>
+      </c>
+      <c r="H355" s="13" t="inlineStr"/>
+      <c r="I355" s="13" t="inlineStr"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I5002">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$A2="☑"</formula>
     </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$A2="☑"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A5002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"☑,☐"</formula1>
+    </dataValidation>
     <dataValidation sqref="A2:A5002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"☑,☐"</formula1>
     </dataValidation>
@@ -16250,6 +16338,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D351" r:id="rId350"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D352" r:id="rId351"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D355" r:id="rId354"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16261,7 +16351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -17416,6 +17506,58 @@
       <c r="H28" s="3" t="inlineStr">
         <is>
           <t>11.08.2026 10:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Ondřej Havelka a jeho Melody Makers / koncert</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>https://polar.cz/kam-vyrazit/moravskoslezsky-kraj/cely-ms-kraj/11000017180/ondrej-havelka-a-jeho-melody-makers--koncert</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr"/>
+      <c r="D29" s="13" t="inlineStr"/>
+      <c r="E29" s="13" t="inlineStr"/>
+      <c r="F29" s="13" t="inlineStr"/>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Jiné</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>11.08.2026 08:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Učitelé praktického vyučování (kromě pro žáky se speciálními vzdělávacími potřebami)</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>https://polar.cz/nabidka-prace/ostrava/detail/33291660710/ucitele-praktickeho-vyucovani-krome-pro-zaky-se-specialnimi-vzdelavacimi-potrebami</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr"/>
+      <c r="E30" s="11" t="inlineStr"/>
+      <c r="F30" s="11" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>Jiné</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>11.08.2026 08:50</t>
         </is>
       </c>
     </row>
@@ -17448,6 +17590,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>